<commit_message>
Kjønn og nasjonalitet på produsent bare på ext
</commit_message>
<xml_diff>
--- a/assets/feltliste.xlsx
+++ b/assets/feltliste.xlsx
@@ -663,7 +663,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">production, production[].type.value.no, production[].person.role.value.no, production[].dateFrom, production[].dateTo, production[].dateFromYear, production[].dateToYear, production[].description.value.no, production[].person.personRef, production[].person.uuid, production[].person._resolved.name, production[].person._resolved.birthYear, production[].person._resolved.deathYear, production[].person._resolved.gender, production[].person._resolved.nationality, production[].person.personCertainty.value.no, production[].place._resolved.name, production[].place.placeType.value.no, production[].place.placeCertainty.value.no</t>
+          <t xml:space="preserve">production, production[].type.value.no, production[].person.role.value.no, production[].dateFrom, production[].dateTo, production[].dateFromYear, production[].dateToYear, production[].description.value.no, production[].person.personRef, production[].person.uuid, production[].person._resolved.name, production[].person._resolved.birthYear, production[].person._resolved.deathYear, production[].person.personCertainty.value.no, production[].place._resolved.name, production[].place.placeType.value.no, production[].place.placeCertainty.value.no</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1134,7 +1134,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">production[].person.gender</t>
+          <t xml:space="preserve">production[].person.certainty</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1144,22 +1144,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">production[].person._resolved.gender</t>
+          <t xml:space="preserve">production[].person.personCertainty.value.no</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">direkte</t>
+          <t xml:space="preserve">språkvalgt verdi</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kjønn (fra personregisteret)</t>
+          <t xml:space="preserve">Sikkerhet for tilskrivningen</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gender (from the person register)</t>
+          <t xml:space="preserve">Certainty of attribution</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1171,81 +1171,81 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">production[].person.nationality</t>
+          <t xml:space="preserve">production[].place</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">liste</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">production[].person._resolved.nationality</t>
+          <t xml:space="preserve">production[].place._resolved.name, production[].place.placeType.value.no, production[].place.placeCertainty.value.no</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">direkte</t>
+          <t xml:space="preserve">avledet (se DATAMODELL_OFFENTLIG.md)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nasjonalitet</t>
+          <t xml:space="preserve">Produksjonssted (navn, type, sikkerhet)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nationality</t>
+          <t xml:space="preserve">Place of production (name, type, certainty)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">nei</t>
+          <t xml:space="preserve">ja</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">production[].person.certainty</t>
+          <t xml:space="preserve">production[].place.name</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">tekst</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">production[].person.personCertainty.value.no</t>
+          <t xml:space="preserve">production[].place._resolved.name</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">språkvalgt verdi</t>
+          <t xml:space="preserve">direkte</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sikkerhet for tilskrivningen</t>
+          <t xml:space="preserve">Stedsnavn fra stedsregisteret</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Certainty of attribution</t>
+          <t xml:space="preserve">Place name from the place register</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">nei</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">production[].place</t>
+          <t xml:space="preserve">production[].place.type</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1255,34 +1255,34 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">production[].place._resolved.name, production[].place.placeType.value.no, production[].place.placeCertainty.value.no</t>
+          <t xml:space="preserve">production[].place.placeType.value.no</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">avledet (se DATAMODELL_OFFENTLIG.md)</t>
+          <t xml:space="preserve">språkvalgt verdi</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Produksjonssted (navn, type, sikkerhet)</t>
+          <t xml:space="preserve">Stedstype, for eksempel Produksjonssted</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Place of production (name, type, certainty)</t>
+          <t xml:space="preserve">Place type, e.g. Place of production</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">ja</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">production[].place.name</t>
+          <t xml:space="preserve">production[].place.certainty</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1292,22 +1292,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">production[].place._resolved.name</t>
+          <t xml:space="preserve">production[].place.placeCertainty.value.no</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">direkte</t>
+          <t xml:space="preserve">språkvalgt verdi</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stedsnavn fra stedsregisteret</t>
+          <t xml:space="preserve">Sikkerhet, for eksempel antatt</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Place name from the place register</t>
+          <t xml:space="preserve">Certainty, e.g. assumed</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1319,106 +1319,106 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">production[].place.type</t>
+          <t xml:space="preserve">materials</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">liste</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">production[].place.placeType.value.no</t>
+          <t xml:space="preserve">materials, materials[].value.no</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">språkvalgt verdi</t>
+          <t xml:space="preserve">liste, språkvalgt</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stedstype, for eksempel Produksjonssted</t>
+          <t xml:space="preserve">Materialer</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Place type, e.g. Place of production</t>
+          <t xml:space="preserve">Materials</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ja</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">production[].place.certainty</t>
+          <t xml:space="preserve">techniques</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">liste</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">production[].place.placeCertainty.value.no</t>
+          <t xml:space="preserve">techniques, techniques[].value.no</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">språkvalgt verdi</t>
+          <t xml:space="preserve">liste, språkvalgt</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sikkerhet, for eksempel antatt</t>
+          <t xml:space="preserve">Teknikker</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Certainty, e.g. assumed</t>
+          <t xml:space="preserve">Techniques</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ja</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">materials</t>
+          <t xml:space="preserve">materialTechniqueDescription</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">liste</t>
+          <t xml:space="preserve">tekst</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">materials, materials[].value.no</t>
+          <t xml:space="preserve">materialTechniqueDescription.no</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">liste, språkvalgt</t>
+          <t xml:space="preserve">språkvalgt verdi</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Materialer</t>
+          <t xml:space="preserve">Materiale og teknikk som fritekst</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Materials</t>
+          <t xml:space="preserve">Material and technique as free text</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1430,7 +1430,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">techniques</t>
+          <t xml:space="preserve">dimensions</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">techniques, techniques[].value.no</t>
+          <t xml:space="preserve">dimensions, dimensions[].type.value.no, dimensions[].value, dimensions[].unit.value.no, dimensions[].category.value.no</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1450,24 +1450,24 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Teknikker</t>
+          <t xml:space="preserve">Mål</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Techniques</t>
+          <t xml:space="preserve">Dimensions</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">ja</t>
+          <t xml:space="preserve">nei (strukturert; nettsiden viser publishableDimensions)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">materialTechniqueDescription</t>
+          <t xml:space="preserve">dimensions[].type</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">materialTechniqueDescription.no</t>
+          <t xml:space="preserve">dimensions[].type.value.no</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1487,61 +1487,61 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Materiale og teknikk som fritekst</t>
+          <t xml:space="preserve">Måltype</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Material and technique as free text</t>
+          <t xml:space="preserve">Type of measurement</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve">ja</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">dimensions</t>
+          <t xml:space="preserve">dimensions[].value</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">liste</t>
+          <t xml:space="preserve">heltall</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">dimensions, dimensions[].type.value.no, dimensions[].value, dimensions[].unit.value.no, dimensions[].category.value.no</t>
+          <t xml:space="preserve">dimensions[].value</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">liste, språkvalgt</t>
+          <t xml:space="preserve">direkte</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mål</t>
+          <t xml:space="preserve">Verdi</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dimensions</t>
+          <t xml:space="preserve">Value</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">nei (strukturert; nettsiden viser publishableDimensions)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">dimensions[].type</t>
+          <t xml:space="preserve">dimensions[].unit</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">dimensions[].type.value.no</t>
+          <t xml:space="preserve">dimensions[].unit.value.no</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1561,12 +1561,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Måltype</t>
+          <t xml:space="preserve">Enhet</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Type of measurement</t>
+          <t xml:space="preserve">Unit</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1578,32 +1578,32 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">dimensions[].value</t>
+          <t xml:space="preserve">dimensions[].category</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">heltall</t>
+          <t xml:space="preserve">tekst</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">dimensions[].value</t>
+          <t xml:space="preserve">dimensions[].category.value.no</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">direkte</t>
+          <t xml:space="preserve">språkvalgt verdi</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verdi</t>
+          <t xml:space="preserve">Kategori</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Value</t>
+          <t xml:space="preserve">Category</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1615,7 +1615,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">dimensions[].unit</t>
+          <t xml:space="preserve">publishableDimensions</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">dimensions[].unit.value.no</t>
+          <t xml:space="preserve">publishableDimensions.no</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1635,24 +1635,24 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enhet</t>
+          <t xml:space="preserve">Mål som tekst for publisering</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unit</t>
+          <t xml:space="preserve">Dimensions as text for publication</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ja</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">dimensions[].category</t>
+          <t xml:space="preserve">collection</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">dimensions[].category.value.no</t>
+          <t xml:space="preserve">collection.value.no</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1672,24 +1672,24 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kategori</t>
+          <t xml:space="preserve">Samling</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Category</t>
+          <t xml:space="preserve">Collection</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">delvis (nettsiden viser også institusjon)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">publishableDimensions</t>
+          <t xml:space="preserve">creditLine</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">publishableDimensions.no</t>
+          <t xml:space="preserve">creditLine.no</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1709,12 +1709,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mål som tekst for publisering</t>
+          <t xml:space="preserve">Kreditering</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dimensions as text for publication</t>
+          <t xml:space="preserve">Credit line</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -1726,69 +1726,69 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">collection</t>
+          <t xml:space="preserve">keywords</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">tekst</t>
+          <t xml:space="preserve">liste</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">collection.value.no</t>
+          <t xml:space="preserve">keywords, keywords[].value.no</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">språkvalgt verdi</t>
+          <t xml:space="preserve">liste, språkvalgt</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Samling</t>
+          <t xml:space="preserve">Emneord fra katalogen</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Collection</t>
+          <t xml:space="preserve">Subject terms from the catalogue</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t xml:space="preserve">delvis (nettsiden viser også institusjon)</t>
+          <t xml:space="preserve">ja</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">creditLine</t>
+          <t xml:space="preserve">motifType</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">tekst</t>
+          <t xml:space="preserve">liste</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">creditLine.no</t>
+          <t xml:space="preserve">motif.type, motif.type[].value.no</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">språkvalgt verdi</t>
+          <t xml:space="preserve">liste, språkvalgt</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kreditering</t>
+          <t xml:space="preserve">Motivtype</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Credit line</t>
+          <t xml:space="preserve">Motif type</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -1800,7 +1800,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">keywords</t>
+          <t xml:space="preserve">classification</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">keywords, keywords[].value.no</t>
+          <t xml:space="preserve">classification, classification[].value.no</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1820,12 +1820,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emneord fra katalogen</t>
+          <t xml:space="preserve">Klassifikasjon</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Subject terms from the catalogue</t>
+          <t xml:space="preserve">Classification</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -1837,32 +1837,32 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">motifType</t>
+          <t xml:space="preserve">owner</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">liste</t>
+          <t xml:space="preserve">tekst</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">motif.type, motif.type[].value.no</t>
+          <t xml:space="preserve">_ownerResolved.name</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">liste, språkvalgt</t>
+          <t xml:space="preserve">direkte</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Motivtype</t>
+          <t xml:space="preserve">Eier</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Motif type</t>
+          <t xml:space="preserve">Owner</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -1874,7 +1874,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">classification</t>
+          <t xml:space="preserve">inscriptions</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">classification, classification[].value.no</t>
+          <t xml:space="preserve">inscriptionsLabels, inscriptionsLabels[].type.value.no, inscriptionsLabels[].transcription.value.no, inscriptionsLabels[].position.value.no, inscriptionsLabels[].method.value.no, inscriptionsLabels[].language.value.no, inscriptionsLabels[].inscriber.value.no, inscriptionsLabels[].date.value.no</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1894,12 +1894,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Klassifikasjon</t>
+          <t xml:space="preserve">Påskrifter, signaturer og stempler</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Classification</t>
+          <t xml:space="preserve">Inscriptions, signatures and stamps</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -1911,7 +1911,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">owner</t>
+          <t xml:space="preserve">inscriptions[].type</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1921,71 +1921,71 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">_ownerResolved.name</t>
+          <t xml:space="preserve">inscriptionsLabels[].type.value.no</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">direkte</t>
+          <t xml:space="preserve">avledet (se DATAMODELL_OFFENTLIG.md)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eier</t>
+          <t xml:space="preserve">Type: Påskrift, Signatur, Stempel …</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Owner</t>
+          <t xml:space="preserve">Type: Inscription, Signature, Stamp …</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t xml:space="preserve">ja</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptions</t>
+          <t xml:space="preserve">inscriptions[].transcription</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">liste</t>
+          <t xml:space="preserve">tekst</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptionsLabels, inscriptionsLabels[].type.value.no, inscriptionsLabels[].transcription.value.no, inscriptionsLabels[].position.value.no, inscriptionsLabels[].method.value.no, inscriptionsLabels[].language.value.no, inscriptionsLabels[].inscriber.value.no, inscriptionsLabels[].date.value.no</t>
+          <t xml:space="preserve">inscriptionsLabels[].transcription.value.no</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">liste, språkvalgt</t>
+          <t xml:space="preserve">avledet (se DATAMODELL_OFFENTLIG.md)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Påskrifter, signaturer og stempler</t>
+          <t xml:space="preserve">Teksten slik den står på verket</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inscriptions, signatures and stamps</t>
+          <t xml:space="preserve">The text as written on the work</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t xml:space="preserve">ja</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptions[].type</t>
+          <t xml:space="preserve">inscriptions[].position</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptionsLabels[].type.value.no</t>
+          <t xml:space="preserve">inscriptionsLabels[].position.value.no</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2005,12 +2005,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Type: Påskrift, Signatur, Stempel …</t>
+          <t xml:space="preserve">Plassering på verket</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Type: Inscription, Signature, Stamp …</t>
+          <t xml:space="preserve">Position on the work</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2022,7 +2022,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptions[].transcription</t>
+          <t xml:space="preserve">inscriptions[].method</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptionsLabels[].transcription.value.no</t>
+          <t xml:space="preserve">inscriptionsLabels[].method.value.no</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2042,12 +2042,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Teksten slik den står på verket</t>
+          <t xml:space="preserve">Teknikk for påskriften</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t xml:space="preserve">The text as written on the work</t>
+          <t xml:space="preserve">Method of the inscription</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2059,7 +2059,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptions[].position</t>
+          <t xml:space="preserve">inscriptions[].language</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptionsLabels[].position.value.no</t>
+          <t xml:space="preserve">inscriptionsLabels[].language.value.no</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2079,12 +2079,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plassering på verket</t>
+          <t xml:space="preserve">Språk</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Position on the work</t>
+          <t xml:space="preserve">Language</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2096,7 +2096,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptions[].method</t>
+          <t xml:space="preserve">inscriptions[].inscriber</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptionsLabels[].method.value.no</t>
+          <t xml:space="preserve">inscriptionsLabels[].inscriber.value.no</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2116,12 +2116,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Teknikk for påskriften</t>
+          <t xml:space="preserve">Hvem som skrev</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Method of the inscription</t>
+          <t xml:space="preserve">Inscriber</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2133,7 +2133,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptions[].language</t>
+          <t xml:space="preserve">inscriptions[].date</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptionsLabels[].language.value.no</t>
+          <t xml:space="preserve">inscriptionsLabels[].date.value.no</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2153,12 +2153,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Språk</t>
+          <t xml:space="preserve">Datering av påskriften</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Language</t>
+          <t xml:space="preserve">Date of the inscription</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2170,44 +2170,44 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptions[].inscriber</t>
+          <t xml:space="preserve">provenance</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">tekst</t>
+          <t xml:space="preserve">liste</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptionsLabels[].inscriber.value.no</t>
+          <t xml:space="preserve">provenanceOwnership, provenanceOwnership[].type.value.no, provenanceOwnership[].owner._resolved.name, provenanceOwnership[].owner.role.value.no, provenanceOwnership[].owner.certainty.value.no, provenanceOwnership[].place._resolved.name, provenanceOwnership[].dateFrom, provenanceOwnership[].dateTo, provenanceOwnership[].dateFromYear, provenanceOwnership[].dateToYear</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">avledet (se DATAMODELL_OFFENTLIG.md)</t>
+          <t xml:space="preserve">liste, språkvalgt</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hvem som skrev</t>
+          <t xml:space="preserve">Proveniens</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inscriber</t>
+          <t xml:space="preserve">Provenance</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ja</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptions[].date</t>
+          <t xml:space="preserve">provenance[].type</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">inscriptionsLabels[].date.value.no</t>
+          <t xml:space="preserve">provenanceOwnership[].type.value.no</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2227,12 +2227,12 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Datering av påskriften</t>
+          <t xml:space="preserve">Type: Eierskap, Aksesjon, Ervervelse …</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Date of the inscription</t>
+          <t xml:space="preserve">Type: Ownership, Accession, Acquisition …</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2244,44 +2244,44 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenance</t>
+          <t xml:space="preserve">provenance[].owner</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">liste</t>
+          <t xml:space="preserve">tekst</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenanceOwnership, provenanceOwnership[].type.value.no, provenanceOwnership[].owner._resolved.name, provenanceOwnership[].owner.role.value.no, provenanceOwnership[].owner.certainty.value.no, provenanceOwnership[].place._resolved.name, provenanceOwnership[].dateFrom, provenanceOwnership[].dateTo, provenanceOwnership[].dateFromYear, provenanceOwnership[].dateToYear</t>
+          <t xml:space="preserve">provenanceOwnership[].owner._resolved.name</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">liste, språkvalgt</t>
+          <t xml:space="preserve">direkte</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proveniens</t>
+          <t xml:space="preserve">Eierens navn fra personregisteret</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Provenance</t>
+          <t xml:space="preserve">Owner's name from the person register</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t xml:space="preserve">ja</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenance[].type</t>
+          <t xml:space="preserve">provenance[].role</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenanceOwnership[].type.value.no</t>
+          <t xml:space="preserve">provenanceOwnership[].owner.role.value.no</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2301,12 +2301,12 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Type: Eierskap, Aksesjon, Ervervelse …</t>
+          <t xml:space="preserve">Rolle, for eksempel [40] Tidligere eier</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Type: Ownership, Accession, Acquisition …</t>
+          <t xml:space="preserve">Role, e.g. [40] Previous owner</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -2318,7 +2318,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenance[].owner</t>
+          <t xml:space="preserve">provenance[].certainty</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2328,22 +2328,22 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenanceOwnership[].owner._resolved.name</t>
+          <t xml:space="preserve">provenanceOwnership[].owner.certainty.value.no</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t xml:space="preserve">direkte</t>
+          <t xml:space="preserve">avledet (se DATAMODELL_OFFENTLIG.md)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eierens navn fra personregisteret</t>
+          <t xml:space="preserve">Sikkerhet</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Owner's name from the person register</t>
+          <t xml:space="preserve">Certainty</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2355,32 +2355,32 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenance[].role</t>
+          <t xml:space="preserve">provenance[].place</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">tekst</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenanceOwnership[].owner.role.value.no</t>
+          <t xml:space="preserve">provenanceOwnership[].place._resolved.name</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t xml:space="preserve">avledet (se DATAMODELL_OFFENTLIG.md)</t>
+          <t xml:space="preserve">direkte</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rolle, for eksempel [40] Tidligere eier</t>
+          <t xml:space="preserve">Sted fra stedsregisteret</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Role, e.g. [40] Previous owner</t>
+          <t xml:space="preserve">Place from the place register</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2392,7 +2392,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenance[].certainty</t>
+          <t xml:space="preserve">provenance[].dateFrom</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2402,22 +2402,22 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenanceOwnership[].owner.certainty.value.no</t>
+          <t xml:space="preserve">provenanceOwnership[].dateFrom</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t xml:space="preserve">avledet (se DATAMODELL_OFFENTLIG.md)</t>
+          <t xml:space="preserve">direkte</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sikkerhet</t>
+          <t xml:space="preserve">Fra (datotekst)</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Certainty</t>
+          <t xml:space="preserve">From (date text)</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2429,17 +2429,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenance[].place</t>
+          <t xml:space="preserve">provenance[].dateTo</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">tekst</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenanceOwnership[].place._resolved.name</t>
+          <t xml:space="preserve">provenanceOwnership[].dateTo</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2449,12 +2449,12 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sted fra stedsregisteret</t>
+          <t xml:space="preserve">Til (datotekst)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Place from the place register</t>
+          <t xml:space="preserve">To (date text)</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2466,17 +2466,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenance[].dateFrom</t>
+          <t xml:space="preserve">provenance[].dateFromYear</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">tekst</t>
+          <t xml:space="preserve">heltall</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenanceOwnership[].dateFrom</t>
+          <t xml:space="preserve">provenanceOwnership[].dateFromYear</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2486,12 +2486,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fra (datotekst)</t>
+          <t xml:space="preserve">Fra år</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t xml:space="preserve">From (date text)</t>
+          <t xml:space="preserve">From year</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2503,17 +2503,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenance[].dateTo</t>
+          <t xml:space="preserve">provenance[].dateToYear</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">tekst</t>
+          <t xml:space="preserve">heltall</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenanceOwnership[].dateTo</t>
+          <t xml:space="preserve">provenanceOwnership[].dateToYear</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2523,12 +2523,12 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Til (datotekst)</t>
+          <t xml:space="preserve">Til år</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t xml:space="preserve">To (date text)</t>
+          <t xml:space="preserve">To year</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2540,54 +2540,54 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenance[].dateFromYear</t>
+          <t xml:space="preserve">copyright</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">heltall</t>
+          <t xml:space="preserve">liste</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenanceOwnership[].dateFromYear</t>
+          <t xml:space="preserve">copyrights, copyrights[]._resolved.name, copyrights[]._managerResolved.name, copyrights[].status.value.no, copyrights[].dateTo</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t xml:space="preserve">direkte</t>
+          <t xml:space="preserve">liste, språkvalgt</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fra år</t>
+          <t xml:space="preserve">Opphavsrett: rettighetshaver, forvalter, status og utløp</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t xml:space="preserve">From year</t>
+          <t xml:space="preserve">Copyright: holder, manager, status and expiry</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ja</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenance[].dateToYear</t>
+          <t xml:space="preserve">copyright[].holder</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">heltall</t>
+          <t xml:space="preserve">tekst</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">provenanceOwnership[].dateToYear</t>
+          <t xml:space="preserve">copyrights[]._resolved.name</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2597,12 +2597,12 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Til år</t>
+          <t xml:space="preserve">Rettighetshaver</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t xml:space="preserve">To year</t>
+          <t xml:space="preserve">Rights holder</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -2614,44 +2614,44 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">copyright</t>
+          <t xml:space="preserve">copyright[].manager</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">liste</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve">copyrights, copyrights[]._resolved.name, copyrights[]._managerResolved.name, copyrights[].status.value.no, copyrights[].dateTo</t>
+          <t xml:space="preserve">copyrights[]._managerResolved.name</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t xml:space="preserve">liste, språkvalgt</t>
+          <t xml:space="preserve">direkte</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opphavsrett: rettighetshaver, forvalter, status og utløp</t>
+          <t xml:space="preserve">Forvalter, for eksempel BONO</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Copyright: holder, manager, status and expiry</t>
+          <t xml:space="preserve">Rights manager, e.g. BONO</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t xml:space="preserve">ja</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">copyright[].holder</t>
+          <t xml:space="preserve">copyright[].status</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2661,22 +2661,22 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve">copyrights[]._resolved.name</t>
+          <t xml:space="preserve">copyrights[].status.value.no</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t xml:space="preserve">direkte</t>
+          <t xml:space="preserve">avledet (se DATAMODELL_OFFENTLIG.md)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rettighetshaver</t>
+          <t xml:space="preserve">Status</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rights holder</t>
+          <t xml:space="preserve">Status</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -2688,17 +2688,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">copyright[].manager</t>
+          <t xml:space="preserve">copyright[].dateTo</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">tekst</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t xml:space="preserve">copyrights[]._managerResolved.name</t>
+          <t xml:space="preserve">copyrights[].dateTo</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2708,12 +2708,12 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Forvalter, for eksempel BONO</t>
+          <t xml:space="preserve">Når vernet går ut</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rights manager, e.g. BONO</t>
+          <t xml:space="preserve">When protection expires</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -2725,91 +2725,91 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">copyright[].status</t>
+          <t xml:space="preserve">publicDomain</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">tekst</t>
+          <t xml:space="preserve">boolsk</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t xml:space="preserve">copyrights[].status.value.no</t>
+          <t xml:space="preserve">publicDomain</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t xml:space="preserve">avledet (se DATAMODELL_OFFENTLIG.md)</t>
+          <t xml:space="preserve">direkte</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Status</t>
+          <t xml:space="preserve">Fri bruk</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Status</t>
+          <t xml:space="preserve">Public domain</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">nei</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">copyright[].dateTo</t>
+          <t xml:space="preserve">multimedia</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">tekst</t>
+          <t xml:space="preserve">liste</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">copyrights[].dateTo</t>
+          <t xml:space="preserve">multimedia[] (bare publiserte bilder)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t xml:space="preserve">direkte</t>
+          <t xml:space="preserve">liste, språkvalgt</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Når vernet går ut</t>
+          <t xml:space="preserve">Publiserte bilder</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t xml:space="preserve">When protection expires</t>
+          <t xml:space="preserve">Published images</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ja (som bildevisning)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">publicDomain</t>
+          <t xml:space="preserve">multimedia[].imageId</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">boolsk</t>
+          <t xml:space="preserve">heltall</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t xml:space="preserve">publicDomain</t>
+          <t xml:space="preserve">multimedia[] (bare publiserte bilder)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2819,12 +2819,12 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fri bruk</t>
+          <t xml:space="preserve">Bildets id (multimediaRef)</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Public domain</t>
+          <t xml:space="preserve">Image id (multimediaRef)</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -2836,12 +2836,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">multimedia</t>
+          <t xml:space="preserve">multimedia[].uuid</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">liste</t>
+          <t xml:space="preserve">tekst</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2851,34 +2851,34 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t xml:space="preserve">liste, språkvalgt</t>
+          <t xml:space="preserve">direkte</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Publiserte bilder</t>
+          <t xml:space="preserve">Bildets UUID</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Published images</t>
+          <t xml:space="preserve">Image UUID</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t xml:space="preserve">ja (som bildevisning)</t>
+          <t xml:space="preserve">nei</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">multimedia[].imageId</t>
+          <t xml:space="preserve">multimedia[].originalFileName</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">heltall</t>
+          <t xml:space="preserve">tekst</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2893,12 +2893,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bildets id (multimediaRef)</t>
+          <t xml:space="preserve">Filnavn i bildearkivet</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Image id (multimediaRef)</t>
+          <t xml:space="preserve">File name in the image archive</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -2910,12 +2910,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">multimedia[].uuid</t>
+          <t xml:space="preserve">multimedia[].thumbnail</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">tekst</t>
+          <t xml:space="preserve">boolsk</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2930,24 +2930,24 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bildets UUID</t>
+          <t xml:space="preserve">Hovedbilde</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Image UUID</t>
+          <t xml:space="preserve">Main image</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t xml:space="preserve">nei</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">multimedia[].originalFileName</t>
+          <t xml:space="preserve">multimedia[].usage</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2967,29 +2967,29 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Filnavn i bildearkivet</t>
+          <t xml:space="preserve">Bruk (Standard-bilde o.l.)</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t xml:space="preserve">File name in the image archive</t>
+          <t xml:space="preserve">Usage</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t xml:space="preserve">nei</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">multimedia[].thumbnail</t>
+          <t xml:space="preserve">multimedia[].photoCredit</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">boolsk</t>
+          <t xml:space="preserve">tekst</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3004,29 +3004,29 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hovedbilde</t>
+          <t xml:space="preserve">Fotograf</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main image</t>
+          <t xml:space="preserve">Photographer</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ja</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">multimedia[].usage</t>
+          <t xml:space="preserve">multimedia[].creditLine</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t xml:space="preserve">tekst</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3036,17 +3036,17 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t xml:space="preserve">direkte</t>
+          <t xml:space="preserve">språkvalgt verdi</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bruk (Standard-bilde o.l.)</t>
+          <t xml:space="preserve">Kreditering for bildet</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usage</t>
+          <t xml:space="preserve">Credit line for the image</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3058,7 +3058,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">multimedia[].photoCredit</t>
+          <t xml:space="preserve">multimedia[].iiifService</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3073,34 +3073,34 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t xml:space="preserve">direkte</t>
+          <t xml:space="preserve">avledet (se DATAMODELL_OFFENTLIG.md)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fotograf</t>
+          <t xml:space="preserve">IIIF Image API-adresse</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Photographer</t>
+          <t xml:space="preserve">IIIF Image API address</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t xml:space="preserve">ja</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">multimedia[].creditLine</t>
+          <t xml:space="preserve">multimedia[].imageUrl</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">tekst</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3110,17 +3110,17 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t xml:space="preserve">språkvalgt verdi</t>
+          <t xml:space="preserve">avledet (se DATAMODELL_OFFENTLIG.md)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kreditering for bildet</t>
+          <t xml:space="preserve">Bilde-URL (1200 px bredde)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Credit line for the image</t>
+          <t xml:space="preserve">Image URL (1200 px wide)</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -3132,17 +3132,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">multimedia[].iiifService</t>
+          <t xml:space="preserve">primaryImage</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t xml:space="preserve">tekst</t>
+          <t xml:space="preserve">objekt</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t xml:space="preserve">multimedia[] (bare publiserte bilder)</t>
+          <t xml:space="preserve">multimedia[] (thumbnail, usage, originalFileName)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -3152,89 +3152,15 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t xml:space="preserve">IIIF Image API-adresse</t>
+          <t xml:space="preserve">Hovedbildet (samme form som multimedia[])</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t xml:space="preserve">IIIF Image API address</t>
+          <t xml:space="preserve">Main image (same shape as multimedia[])</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">multimedia[].imageUrl</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tekst</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">multimedia[] (bare publiserte bilder)</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">avledet (se DATAMODELL_OFFENTLIG.md)</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bilde-URL (1200 px bredde)</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Image URL (1200 px wide)</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">primaryImage</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">objekt</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">multimedia[] (thumbnail, usage, originalFileName)</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">avledet (se DATAMODELL_OFFENTLIG.md)</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hovedbildet (samme form som multimedia[])</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Main image (same shape as multimedia[])</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
         <is>
           <t xml:space="preserve">ja (som bildevisning)</t>
         </is>

</xml_diff>

<commit_message>
Eksempelsvar, feltsider med eksempel og kilde, ext og full, endringslogg, avviklede endepunkter, sidestørrelser og mellomlagring
</commit_message>
<xml_diff>
--- a/assets/feltliste.xlsx
+++ b/assets/feltliste.xlsx
@@ -57,6 +57,11 @@
           <t xml:space="preserve">på Samlingen på nett</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eksempel</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -94,6 +99,11 @@
           <t xml:space="preserve">ja (i adressen)</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NG.M.00939</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -131,6 +141,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NG.M.00939</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -168,6 +183,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C88BFBE7-645D-4EE4-922C-4A3AFA7087F7</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -205,6 +225,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -242,6 +267,11 @@
           <t xml:space="preserve">nei (nettsiden viser labelDate)</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -279,6 +309,11 @@
           <t xml:space="preserve">nei (nettsiden viser labelDate)</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -316,6 +351,11 @@
           <t xml:space="preserve">ja (tom tittel: nettsiden viser betegnelsen)</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Skrik</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -353,6 +393,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Scream</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -390,6 +435,11 @@
           <t xml:space="preserve">delvis (uten type og datoer)</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{title, type, language, dateFrom, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -427,6 +477,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Skrik</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -464,6 +519,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">anvendt</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -501,6 +561,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Norsk</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -538,6 +603,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -575,6 +645,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -612,6 +687,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maleri</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -649,6 +729,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -686,6 +771,11 @@
           <t xml:space="preserve">delvis</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{type, role, dateFrom, dateTo, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -723,6 +813,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Produsert</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -760,6 +855,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kunstner</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -797,6 +897,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -834,6 +939,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -871,6 +981,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -908,6 +1023,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -945,6 +1065,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -982,6 +1107,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">56154</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1019,6 +1149,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">281F289C-1A53-4727-86F8-A335CB4AB072</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1056,6 +1191,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edvard Munch</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1093,6 +1233,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1863</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1130,6 +1275,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1944</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1167,6 +1317,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sikker</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1204,6 +1359,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name, type, certainty}</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1241,6 +1401,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vestlandet (Norge)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1278,6 +1443,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Produksjonssted</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1315,6 +1485,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">antatt</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1352,6 +1527,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Papplate</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1389,6 +1569,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tempera, Fettstift</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1426,6 +1611,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tempera og fettstift på papplate</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1463,6 +1653,11 @@
           <t xml:space="preserve">nei (strukturert; nettsiden viser publishableDimensions)</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{type, value, unit, category}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1500,6 +1695,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bredde</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1537,6 +1737,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">73.5</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1574,6 +1779,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1611,6 +1821,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hovedmål</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1648,6 +1863,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">91 x 73,5 cm</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1685,6 +1905,11 @@
           <t xml:space="preserve">delvis (nettsiden viser også institusjon)</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Billedkunstsamlingene</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1722,6 +1947,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gave fra Olaf Schou 1910</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1759,6 +1989,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bildende kunst</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1796,6 +2031,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Landskap, Portrett</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1833,6 +2073,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">532 - Bildende kunst</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1870,6 +2115,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nasjonalmuseet for kunst, arkitektur og design</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1907,6 +2157,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{type, transcription, position, method, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1944,6 +2199,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Signatur og datering</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1981,6 +2241,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E. Munch 1893</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2018,6 +2283,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nede venstre</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2055,6 +2325,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2092,6 +2367,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2129,6 +2409,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2166,6 +2451,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2203,6 +2493,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{type, owner, role, certainty, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2240,6 +2535,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aksesjon</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2277,6 +2577,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Olaf Schou</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2314,6 +2619,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[20] Giver/siste eier</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2351,6 +2661,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sikker</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2388,6 +2703,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Elmholt Allé 13, Oslo (fylke) (Norge)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2425,6 +2745,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1910</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2462,6 +2787,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1910</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2499,6 +2829,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1910</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2536,6 +2871,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1910</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2573,6 +2913,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{holder, manager, status, dateTo}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2610,6 +2955,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jakob Weidemann</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2647,6 +2997,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BONO</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2684,6 +3039,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aktiv</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2721,6 +3081,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2071-01-01T00.00.00</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2758,6 +3123,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2795,6 +3165,11 @@
           <t xml:space="preserve">ja (som bildevisning)</t>
         </is>
       </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{imageId, uuid, originalFileName, thumbnail, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2832,6 +3207,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43925</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2869,6 +3249,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1040531</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2906,6 +3291,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">54318.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2943,6 +3333,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2980,6 +3375,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detaljbilde</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3017,6 +3417,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Børre Høstland</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3054,6 +3459,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3091,6 +3501,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://ms01.nasjonalmuseet.no/iiif/tif/54318.tif</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3128,6 +3543,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://ms01.nasjonalmuseet.no/iiif/tif/54318.tif/full/12…</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3163,6 +3583,11 @@
       <c r="G85" t="inlineStr">
         <is>
           <t xml:space="preserve">ja (som bildevisning)</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{imageId, uuid, originalFileName, thumbnail, …}</t>
         </is>
       </c>
     </row>
@@ -3218,6 +3643,11 @@
           <t xml:space="preserve">på Samlingen på nett</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eksempel</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3255,6 +3685,11 @@
           <t xml:space="preserve">ja (i adressen)</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NG.M.00939</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3292,6 +3727,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NG.M.00939</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3329,6 +3769,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C88BFBE7-645D-4EE4-922C-4A3AFA7087F7</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3366,6 +3811,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3403,6 +3853,11 @@
           <t xml:space="preserve">nei (nettsiden viser labelDate)</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3440,6 +3895,11 @@
           <t xml:space="preserve">nei (nettsiden viser labelDate)</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3477,6 +3937,11 @@
           <t xml:space="preserve">ja (tom tittel: nettsiden viser betegnelsen)</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Skrik</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3514,6 +3979,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Scream</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3551,6 +4021,11 @@
           <t xml:space="preserve">delvis (uten type og datoer)</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{title, type, language, dateFrom, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3588,6 +4063,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Skrik</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3625,6 +4105,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">anvendt</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3662,6 +4147,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Norsk</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3699,6 +4189,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3736,6 +4231,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3773,6 +4273,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maleri</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3810,6 +4315,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3847,6 +4357,11 @@
           <t xml:space="preserve">delvis</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{type, role, dateFrom, dateTo, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3884,6 +4399,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Produsert</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3921,6 +4441,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kunstner</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3958,6 +4483,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3995,6 +4525,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4032,6 +4567,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4069,6 +4609,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4106,6 +4651,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4143,6 +4693,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">56154</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4180,6 +4735,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">281F289C-1A53-4727-86F8-A335CB4AB072</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4217,6 +4777,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edvard Munch</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4254,6 +4819,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1863</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4291,6 +4861,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1944</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4328,6 +4903,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Male</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4365,6 +4945,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Norway</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4402,6 +4987,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sikker</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4439,6 +5029,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name, type, certainty}</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4476,6 +5071,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vestlandet (Norge)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4513,6 +5113,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Produksjonssted</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4550,6 +5155,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">antatt</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4587,6 +5197,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Papplate</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4624,6 +5239,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tempera, Fettstift</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4661,6 +5281,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tempera og fettstift på papplate</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4698,6 +5323,11 @@
           <t xml:space="preserve">nei (strukturert; nettsiden viser publishableDimensions)</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{type, value, unit, category}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4735,6 +5365,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bredde</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4772,6 +5407,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">73.5</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4809,6 +5449,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4846,6 +5491,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hovedmål</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4883,6 +5533,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">91 x 73,5 cm</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4920,6 +5575,11 @@
           <t xml:space="preserve">delvis (nettsiden viser også institusjon)</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Billedkunstsamlingene</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4957,6 +5617,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gave fra Olaf Schou 1910</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4994,6 +5659,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bildende kunst</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5031,6 +5701,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Landskap, Portrett</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5068,6 +5743,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">532 - Bildende kunst</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5105,6 +5785,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nasjonalmuseet for kunst, arkitektur og design</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5142,6 +5827,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{type, transcription, position, method, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5179,6 +5869,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Signatur og datering</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5216,6 +5911,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E. Munch 1893</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5253,6 +5953,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nede venstre</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5290,6 +5995,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5327,6 +6037,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5364,6 +6079,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5401,6 +6121,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5438,6 +6163,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{type, owner, role, certainty, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5475,6 +6205,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aksesjon</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5512,6 +6247,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Olaf Schou</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5549,6 +6289,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[20] Giver/siste eier</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5586,6 +6331,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sikker</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5623,6 +6373,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Elmholt Allé 13, Oslo (fylke) (Norge)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5660,6 +6415,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1910</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5697,6 +6457,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1910</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5734,6 +6499,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1910</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5771,6 +6541,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1910</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5808,6 +6583,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{holder, manager, status, dateTo}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5845,6 +6625,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jakob Weidemann</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5882,6 +6667,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BONO</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5919,6 +6709,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aktiv</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5956,6 +6751,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2071-01-01T00.00.00</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5993,6 +6793,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6030,6 +6835,11 @@
           <t xml:space="preserve">ja (som bildevisning)</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{imageId, uuid, originalFileName, thumbnail, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6067,6 +6877,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43925</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6104,6 +6919,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1040531</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6141,6 +6961,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">54318.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6178,6 +7003,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6215,6 +7045,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detaljbilde</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6252,6 +7087,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Børre Høstland</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6289,6 +7129,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6326,6 +7171,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://ms01.nasjonalmuseet.no/iiif/tif/54318.tif</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6363,6 +7213,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://ms01.nasjonalmuseet.no/iiif/tif/54318.tif/full/12…</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6400,6 +7255,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{keywords, groups}</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6437,6 +7297,11 @@
           <t xml:space="preserve">nei (skrevet av berikelsen)</t>
         </is>
       </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Papplate, Tempera, Fettstift, …</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6474,6 +7339,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">723af58e-25bd-425d-8a5d-2ed8ff80d530</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6511,6 +7381,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6548,6 +7423,11 @@
           <t xml:space="preserve">ja (som bildevisning)</t>
         </is>
       </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{imageId, uuid, originalFileName, thumbnail, …}</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6585,6 +7465,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -6622,6 +7507,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -6659,6 +7549,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -6696,6 +7591,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -6733,6 +7633,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -6770,6 +7675,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6807,6 +7717,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Billedkunst</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6844,6 +7759,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ART</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -6881,6 +7801,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -6918,6 +7843,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -6953,6 +7883,11 @@
       <c r="G102" t="inlineStr">
         <is>
           <t xml:space="preserve">ja («Utstilt i»)</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{active, room, exhibition, dateFrom, …}</t>
         </is>
       </c>
     </row>
@@ -7008,6 +7943,11 @@
           <t xml:space="preserve">på Samlingen på nett</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eksempel</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7045,6 +7985,11 @@
           <t xml:space="preserve">ja (i adressen)</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NG.M.00939</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7082,6 +8027,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NG.M.00939</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7119,6 +8069,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C88BFBE7-645D-4EE4-922C-4A3AFA7087F7</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7156,6 +8111,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -7193,6 +8153,11 @@
           <t xml:space="preserve">nei (nettsiden viser labelDate)</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -7230,6 +8195,11 @@
           <t xml:space="preserve">nei (nettsiden viser labelDate)</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7267,6 +8237,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ART</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7304,6 +8279,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7341,6 +8321,11 @@
           <t xml:space="preserve">ja (tom tittel: nettsiden viser betegnelsen)</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Skrik</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7378,6 +8363,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Scream, Verzweiflung (Fortvilelse), Verzweiflung</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7415,6 +8405,11 @@
           <t xml:space="preserve">delvis (uten type og datoer)</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{title, type, language, dateFrom, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7452,6 +8447,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Skrik</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7489,6 +8489,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">anvendt</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7526,6 +8531,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Norsk</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7563,6 +8573,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7600,6 +8615,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7637,6 +8657,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maleri</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7674,6 +8699,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Billedkunst</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7711,6 +8741,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7748,6 +8783,11 @@
           <t xml:space="preserve">delvis</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{type, role, dateFrom, dateTo, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7785,6 +8825,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Produsert</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7822,6 +8867,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kunstner</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7859,6 +8909,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7896,6 +8951,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7933,6 +8993,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7970,6 +9035,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1893</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8007,6 +9077,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -8044,6 +9119,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">56154</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -8081,6 +9161,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">281F289C-1A53-4727-86F8-A335CB4AB072</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -8118,6 +9203,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edvard Munch</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -8155,6 +9245,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1863</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -8192,6 +9287,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1944</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8229,6 +9329,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Male</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8266,6 +9371,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Norway</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8303,6 +9413,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sikker</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8340,6 +9455,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{name, type, certainty}</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8377,6 +9497,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vestlandet (Norge)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8414,6 +9539,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Produksjonssted</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -8451,6 +9581,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">antatt</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -8488,6 +9623,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Papplate</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -8525,6 +9665,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tempera, Fettstift</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -8562,6 +9707,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tempera og fettstift på papplate</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -8599,6 +9749,11 @@
           <t xml:space="preserve">nei (strukturert; nettsiden viser publishableDimensions)</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{type, value, unit, category}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -8636,6 +9791,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bredde</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -8673,6 +9833,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">73.5</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -8710,6 +9875,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8747,6 +9917,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hovedmål</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -8784,6 +9959,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">91 x 73,5 cm</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -8821,6 +10001,11 @@
           <t xml:space="preserve">delvis (nettsiden viser også institusjon)</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Billedkunstsamlingene</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -8858,6 +10043,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gave fra Olaf Schou 1910</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -8895,6 +10085,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bildende kunst</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -8932,6 +10127,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Landskap, Portrett</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -8969,6 +10169,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">532 - Bildende kunst</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9006,6 +10211,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nasjonalmuseet for kunst, arkitektur og design</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -9043,6 +10253,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{type, transcription, position, method, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -9080,6 +10295,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Signatur og datering</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -9117,6 +10337,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E. Munch 1893</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -9154,6 +10379,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nede venstre</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -9191,6 +10421,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -9228,6 +10463,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -9265,6 +10505,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -9302,6 +10547,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -9339,6 +10589,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{type, owner, role, certainty, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -9376,6 +10631,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aksesjon</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -9413,6 +10673,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Olaf Schou</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -9450,6 +10715,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[20] Giver/siste eier</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -9487,6 +10757,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sikker</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -9524,6 +10799,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Elmholt Allé 13, Oslo (fylke) (Norge)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -9561,6 +10841,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1910</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -9598,6 +10883,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1910</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -9635,6 +10925,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1910</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -9672,6 +10967,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1910</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -9709,6 +11009,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{holder, manager, status, dateTo}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -9746,6 +11051,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jakob Weidemann</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -9783,6 +11093,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BONO</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -9820,6 +11135,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aktiv</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -9857,6 +11177,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2071-01-01T00.00.00</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -9894,6 +11219,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -9931,6 +11261,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -9968,6 +11303,11 @@
           <t xml:space="preserve">ja (som bildevisning)</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{imageId, uuid, originalFileName, thumbnail, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -10005,6 +11345,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43925</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -10042,6 +11387,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1040531</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -10079,6 +11429,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">54318.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -10116,6 +11471,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">False</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -10153,6 +11513,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detaljbilde</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -10190,6 +11555,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Børre Høstland</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -10227,6 +11597,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -10264,6 +11639,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://ms01.nasjonalmuseet.no/iiif/tif/54318.tif</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -10301,6 +11681,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://ms01.nasjonalmuseet.no/iiif/tif/54318.tif/full/12…</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -10338,6 +11723,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{keywords, groups}</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -10375,6 +11765,11 @@
           <t xml:space="preserve">nei (skrevet av berikelsen)</t>
         </is>
       </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Papplate, Tempera, Fettstift, …</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -10412,6 +11807,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">723af58e-25bd-425d-8a5d-2ed8ff80d530</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -10449,6 +11849,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -10486,6 +11891,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">True</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -10523,6 +11933,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fotostation</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -10560,6 +11975,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{status, source, attempts, lastError, …}</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -10597,6 +12017,11 @@
           <t xml:space="preserve">ja (som bildevisning)</t>
         </is>
       </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{imageId, uuid, originalFileName, thumbnail, …}</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -10634,6 +12059,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{exhibitionID, registrarID, _resolved, publishable}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -10671,6 +12101,11 @@
           <t xml:space="preserve">delvis (motivtype)</t>
         </is>
       </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{keywords, type, classification, description, …}</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -10708,6 +12143,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{sort, type, subtype, primarySecondary, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -10745,6 +12185,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{relevance, literatureRef, pageRef, chicagoCitation, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -10782,6 +12227,11 @@
           <t xml:space="preserve">ja</t>
         </is>
       </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[{managerRef, personRef, status, dateTo, …}, …]</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -10819,6 +12269,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{value, editionNumber, editionNote}</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -10856,6 +12311,11 @@
           <t xml:space="preserve">delvis</t>
         </is>
       </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{dateFrom, dateFromIso, dateFromBegin, dateFromEnd, …}</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -10893,6 +12353,11 @@
           <t xml:space="preserve">nei</t>
         </is>
       </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -10930,6 +12395,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -10965,6 +12435,11 @@
       <c r="G108" t="inlineStr">
         <is>
           <t xml:space="preserve">ja («Utstilt i»)</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{active, room, exhibition, registrarId, …}</t>
         </is>
       </c>
     </row>

</xml_diff>